<commit_message>
benchmark and new input file
</commit_message>
<xml_diff>
--- a/Files/Inputs.xlsx
+++ b/Files/Inputs.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,15 +15,25 @@
     <sheet name="Realtime state" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -35,7 +45,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -45,14 +62,45 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -129,10 +177,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -170,69 +218,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -256,54 +306,53 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -313,7 +362,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -322,7 +371,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -331,7 +380,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -339,10 +388,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -371,7 +420,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -384,13 +433,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
+                <a:tint val="80000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -410,1376 +458,1397 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="3" max="3"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Required columns</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Used in</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="17.25" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Settings</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Global model settings</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>field, value</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>day_ahead and real_time</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Set timestep_minutes here and also pass input.timestep_minutes in the API payload.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="17.25" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Buses</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Fleet battery capacity by vehicle</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>bus_id, bus_kwh, initial_soc</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>day_ahead and real_time</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>initial_soc is optional; this workbook currently sets all buses to 35 for feasibility testing.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="17.25" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Chargers</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Charging asset data in physical units</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>charger_id, charger_kw, max_power_kw</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>day_ahead and real_time</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>The app converts charger_kw to kWh per step using timestep_minutes.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="17.25" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Trips</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Trip schedule and energy need</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>trip_id, bus_id, time_begin, time_end, energy_kwhkm, average_velocity_kmh</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>day_ahead and real_time</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>time_begin and time_end should be written as HH:MM. This template now contains exactly 8 trips.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="17.25" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Prices</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Energy price by timestep</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>timestep, spot_market</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>day_ahead and real_time</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Keep the full day here. If timestep_minutes is omitted in the API, the app can infer it from the daily horizon length.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="17.25" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Realtime state</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Observed fleet state at the current timestep</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>current_timestep, bus_id, current_soc or current_energy_kwh, operation_status, delay_minutes</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>real_time only</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>If operation_status is in_trip, the app resets that trip start to current_timestep. delay_minutes extends the scheduled trip end before the horizon is trimmed.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>API request</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Suggested request payload</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>optimization_mode, current_timestep, input, price_guidance, disturbances</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>API</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Trips can be sent with HH:MM strings. max_iter is not used anymore and should not be sent.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="3" max="3"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="17.25" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>timestep_minutes</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Global discretization in minutes. The app converts charger power and trip energy to kWh per step from this value.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="17.25" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>optimization_mode</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>day_ahead</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Use day_ahead for full-horizon optimization or real_time for rolling optimization from current_timestep onward.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>bus_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>bus_kwh</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>initial_soc</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="17.25" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C2" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="C2" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" ht="17.25" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C3" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="C3" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C4" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="C4" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C5" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="C5" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" ht="17.25" customHeight="1">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C6" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="C6" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" ht="17.25" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C7" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+      <c r="C7" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C8" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
+      <c r="C8" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="17.25" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="C9" t="n">
-        <v>35</v>
+      <c r="C9" s="3" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>charger_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>charger_kw</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>max_power_kw</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    </row>
+    <row r="2" ht="17.25" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C2" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+    </row>
+    <row r="3" ht="17.25" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C3" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+    </row>
+    <row r="4" ht="17.25" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C4" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+    </row>
+    <row r="5" ht="17.25" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C5" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+    </row>
+    <row r="6" ht="17.25" customHeight="1">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C6" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+    </row>
+    <row r="7" ht="17.25" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C7" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+    </row>
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C8" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
+    </row>
+    <row r="9" ht="17.25" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C9" t="n">
-        <v>360</v>
-      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="3" max="3"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="8" min="5" max="5"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>trip_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>bus_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>time_begin</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>time_end</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>energy_kwhkm</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>average_velocity_kmh</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="17.25" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="7" t="n">
         <v>0.923</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" ht="17.25" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>06:00</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>23:00</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="7" t="n">
         <v>0.859</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" ht="17.25" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>05:30</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="7" t="n">
         <v>0.886</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" ht="17.25" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>06:00</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="7" t="n">
         <v>0.88</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
+    <row r="6" ht="17.25" customHeight="1">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.861</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="3" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
+    <row r="7" ht="17.25" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="7" t="n">
         <v>0.891</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="3" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="7" t="n">
         <v>0.923</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="3" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" ht="17.25" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="7" t="n">
         <v>0.903</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="3" t="n">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>timestep</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>spot_market</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="17.25" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="7" t="n">
         <v>0.09619637602179835</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" ht="17.25" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="7" t="n">
         <v>0.09619637602179835</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" ht="17.25" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="7" t="n">
         <v>0.08876599455040872</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" ht="17.25" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.08876599455040872</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
+    <row r="6" ht="17.25" customHeight="1">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.08449662125340598</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
+    <row r="7" ht="17.25" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="7" t="n">
         <v>0.08449662125340598</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="7" t="n">
         <v>0.08228021798365123</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" ht="17.25" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="7" t="n">
         <v>0.08228021798365123</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
+    <row r="10" ht="17.25" customHeight="1">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="7" t="n">
         <v>0.08080803814713895</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="n">
+    <row r="11" ht="17.25" customHeight="1">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="7" t="n">
         <v>0.08080803814713895</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="n">
+    <row r="12" ht="17.25" customHeight="1">
+      <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="7" t="n">
         <v>0.08383324250681198</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
+    <row r="13" ht="17.25" customHeight="1">
+      <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="7" t="n">
         <v>0.08383324250681198</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
+    <row r="14" ht="17.25" customHeight="1">
+      <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="7" t="n">
         <v>0.09252626702997276</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="n">
+    <row r="15" ht="17.25" customHeight="1">
+      <c r="A15" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="7" t="n">
         <v>0.09252626702997276</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
+    <row r="16" ht="17.25" customHeight="1">
+      <c r="A16" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="7" t="n">
         <v>0.102791280653951</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="n">
+    <row r="17" ht="17.25" customHeight="1">
+      <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="7" t="n">
         <v>0.102791280653951</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="n">
+    <row r="18" ht="17.25" customHeight="1">
+      <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="7" t="n">
         <v>0.105717166212534</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="n">
+    <row r="19" ht="17.25" customHeight="1">
+      <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="7" t="n">
         <v>0.105717166212534</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="n">
+    <row r="20" ht="17.25" customHeight="1">
+      <c r="A20" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="7" t="n">
         <v>0.09572980926430517</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="n">
+    <row r="21" ht="17.25" customHeight="1">
+      <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="7" t="n">
         <v>0.09572980926430517</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="n">
+    <row r="22" ht="17.25" customHeight="1">
+      <c r="A22" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="7" t="n">
         <v>0.08299574931880109</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="n">
+    <row r="23" ht="17.25" customHeight="1">
+      <c r="A23" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="7" t="n">
         <v>0.08299574931880109</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="n">
+    <row r="24" ht="17.25" customHeight="1">
+      <c r="A24" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="7" t="n">
         <v>0.077228310626703</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="n">
+    <row r="25" ht="17.25" customHeight="1">
+      <c r="A25" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="7" t="n">
         <v>0.077228310626703</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="n">
+    <row r="26" ht="17.25" customHeight="1">
+      <c r="A26" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="7" t="n">
         <v>0.07437686648501363</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="n">
+    <row r="27" ht="17.25" customHeight="1">
+      <c r="A27" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="7" t="n">
         <v>0.07437686648501363</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="n">
+    <row r="28" ht="17.25" customHeight="1">
+      <c r="A28" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="7" t="n">
         <v>0.07192795640326977</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="n">
+    <row r="29" ht="17.25" customHeight="1">
+      <c r="A29" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="7" t="n">
         <v>0.07192795640326977</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="n">
+    <row r="30" ht="17.25" customHeight="1">
+      <c r="A30" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="7" t="n">
         <v>0.06861103542234331</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="n">
+    <row r="31" ht="17.25" customHeight="1">
+      <c r="A31" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="7" t="n">
         <v>0.06861103542234331</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="n">
+    <row r="32" ht="17.25" customHeight="1">
+      <c r="A32" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="7" t="n">
         <v>0.06739891008174388</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="n">
+    <row r="33" ht="17.25" customHeight="1">
+      <c r="A33" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="7" t="n">
         <v>0.06739891008174388</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="n">
+    <row r="34" ht="17.25" customHeight="1">
+      <c r="A34" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="7" t="n">
         <v>0.07101792915531335</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="n">
+    <row r="35" ht="17.25" customHeight="1">
+      <c r="A35" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="7" t="n">
         <v>0.07101792915531335</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="n">
+    <row r="36" ht="17.25" customHeight="1">
+      <c r="A36" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="7" t="n">
         <v>0.08115062670299727</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="n">
+    <row r="37" ht="17.25" customHeight="1">
+      <c r="A37" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="7" t="n">
         <v>0.08115062670299727</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="n">
+    <row r="38" ht="17.25" customHeight="1">
+      <c r="A38" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="7" t="n">
         <v>0.09418119891008175</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="n">
+    <row r="39" ht="17.25" customHeight="1">
+      <c r="A39" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="7" t="n">
         <v>0.09418119891008175</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="n">
+    <row r="40" ht="17.25" customHeight="1">
+      <c r="A40" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="7" t="n">
         <v>0.1104535694822888</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="n">
+    <row r="41" ht="17.25" customHeight="1">
+      <c r="A41" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="7" t="n">
         <v>0.1104535694822888</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="n">
+    <row r="42" ht="17.25" customHeight="1">
+      <c r="A42" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="7" t="n">
         <v>0.1221265940054496</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="n">
+    <row r="43" ht="17.25" customHeight="1">
+      <c r="A43" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="7" t="n">
         <v>0.1221265940054496</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="n">
+    <row r="44" ht="17.25" customHeight="1">
+      <c r="A44" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="7" t="n">
         <v>0.120581825613079</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="n">
+    <row r="45" ht="17.25" customHeight="1">
+      <c r="A45" s="3" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="7" t="n">
         <v>0.120581825613079</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="n">
+    <row r="46" ht="17.25" customHeight="1">
+      <c r="A46" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="7" t="n">
         <v>0.1114515803814714</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="n">
+    <row r="47" ht="17.25" customHeight="1">
+      <c r="A47" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="7" t="n">
         <v>0.1114515803814714</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="n">
+    <row r="48" ht="17.25" customHeight="1">
+      <c r="A48" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="7" t="n">
         <v>0.1015224043715847</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="n">
+    <row r="49" ht="17.25" customHeight="1">
+      <c r="A49" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="7" t="n">
         <v>0.1015224043715847</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14.43357142857143" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="5" min="5" max="5"/>
+    <col width="12.43357142857143" bestFit="1" customWidth="1" style="4" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>current_timestep</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>bus_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>current_soc</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>current_energy_kwh</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>operation_status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>delay_minutes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="17.25" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>in_trip</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>idle</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" ht="17.25" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>idle</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" ht="17.25" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>idle</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" ht="17.25" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>idle</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
+    <row r="6" ht="17.25" customHeight="1">
+      <c r="A6" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>idle</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="3" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
+    <row r="7" ht="17.25" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>idle</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="3" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>idle</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="3" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" ht="17.25" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>idle</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="3" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>